<commit_message>
Added a menu version of scheduleGen
</commit_message>
<xml_diff>
--- a/src/scheduleResponse/Schedule.xlsx
+++ b/src/scheduleResponse/Schedule.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Desen(Jucemar)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -473,12 +473,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Geogr(Pedro)</t>
+          <t>Geogr(Zeca)</t>
         </is>
       </c>
     </row>
@@ -490,22 +490,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PPW(Jessica)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>PVIDA(Adriana)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Filos(Alex)</t>
+          <t>Geogr(Zeca)</t>
         </is>
       </c>
     </row>
@@ -517,22 +517,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fisic(Maria Alice)</t>
+          <t>PPW(Jessica)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>PVIDA(Adriana)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Filos(Alex)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lingu(Gabriel)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Ingle(Natalia)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Artes(Joice)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Desen(Lucas)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
     </row>
@@ -571,27 +571,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Progr(Gabriel)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Artes(Joice)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Filos(Alex)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Model(Jessica)</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Matem(Bernardo)</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>INTERVALO</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
@@ -600,135 +604,135 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7h45</t>
+          <t>13h15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Matem(Silvana)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Matem(Bernardo)</t>
+          <t>Ed fi(Xuxa)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ed fi(MaitÃª)</t>
+          <t>Filos(Alex)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8h30</t>
+          <t>14h00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Siste(Eloy)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Progr(Gabriel)</t>
+          <t>Ed fi(Xuxa)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Filos(Alex)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>Artes(Joice)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>9h15</t>
+          <t>14h45</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Siste(Eloy)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Progr(Gabriel)</t>
+          <t>Filos(Alex)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Filos(Alex)</t>
+          <t>Ed fi(Xuxa)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>Artes(Joice)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10h15</t>
+          <t>15h45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>Ed fi(Xuxa)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Filos(Alex)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Matem(Silvana)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>PPW(Jessica)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11h00</t>
+          <t>16h30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>Ed fi(Xuxa)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Socio(Tarso)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Lingu(Evandro)</t>
         </is>
       </c>
     </row>
@@ -747,22 +751,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>Artes(Joice)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>PPW(Jessica)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Biolo(Debora)</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Lingu(Gabriel)</t>
-        </is>
-      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Socio(Tarso)</t>
         </is>
       </c>
     </row>
@@ -774,22 +778,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Model(Jessica)</t>
+          <t>Artes(Joice)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ingle(Natalia)</t>
+          <t>Portu(Marcia)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Progr(Gabriel)</t>
+          <t>PPW(Jessica)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Siste(Isabela)</t>
+          <t>Socio(Tarso)</t>
         </is>
       </c>
     </row>
@@ -801,22 +805,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>PVIDA(Adriana)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ingle(Natalia)</t>
+          <t>Artes(Joice)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>PPW(Jessica)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Filos(Alex)</t>
         </is>
       </c>
     </row>
@@ -828,22 +832,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>PVIDA(Adriana)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>Artes(Joice)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Lingu(Evandro)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Progr(Gabriel)</t>
+          <t>Filos(Alex)</t>
         </is>
       </c>
     </row>
@@ -855,27 +859,31 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>PPW(Jessica)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>Filos(Alex)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Lingu(Gabriel)</t>
+          <t>PVIDA(Adriana)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>INTERVALO</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
@@ -884,135 +892,135 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7h45</t>
+          <t>13h15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ingle(Natalia)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>PPW(Jessica)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Ed fi(MaitÃª)</t>
+          <t>Filos(Alex)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>PPW(Jessica)</t>
+          <t>PVIDA(Adriana)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>8h30</t>
+          <t>14h00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ingle(Natalia)</t>
+          <t>Biolo(Debora)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>Lingu(Evandro)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Geogr(Pedro)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Model(Jessica)</t>
+          <t>Quimi(Karina)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9h15</t>
+          <t>14h45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ed fi(MaitÃª)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Geogr(Pedro)</t>
+          <t>Lingu(Evandro)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>Siste(Eloy)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10h15</t>
+          <t>15h45</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Desen(Lucas)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Geogr(Zeca)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Progr(Gabriel)</t>
+          <t>Quimi(Karina)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>Siste(Eloy)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11h00</t>
+          <t>16h30</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Geogr(Pedro)</t>
+          <t>Socio(Tarso)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Geogr(Zeca)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Socio(Manuela)</t>
+          <t>Ingle(Natalia)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ingle(Natalia)</t>
+          <t>Desen(Jucemar)</t>
         </is>
       </c>
     </row>
@@ -1031,22 +1039,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Teste(Edilson)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Fisic(Maria Alice)</t>
+          <t>Portu(Marcia)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Progr(Gabriel)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
     </row>
@@ -1058,22 +1066,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Filos(Alex)</t>
+          <t>Teste(Edilson)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ingle(Natalia)</t>
+          <t>Portu(Marcia)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
     </row>
@@ -1085,22 +1093,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Filos(Alex)</t>
+          <t>Artes(Joice)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fisic(Maria Alice)</t>
+          <t>PPW(Jessica)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ingle(Natalia)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Biolo(Debora)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
     </row>
@@ -1112,22 +1120,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>Socio(Tarso)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Desen(Lucas)</t>
+          <t>Model(Jessica)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Histo(Arthur)</t>
+          <t>Fisic(Felipe)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fisic(Maria Alice)</t>
+          <t>Progr(Evandro)</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1147,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Teste(Heitor)</t>
+          <t>Socio(Tarso)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ed fi(MaitÃª)</t>
+          <t>PVIDA(Adriana)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1154,7 +1162,729 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>Histo(Walbert)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>INTERVALO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13h15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PVIDA(Adriana)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Artes(Joice)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PPW(Jessica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14h00</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Model(Jessica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>14h45</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Ed fi(Xuxa)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15h45</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Socio(Tarso)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ed fi(Xuxa)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16h30</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Socio(Tarso)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Lingu(Evandro)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Ed fi(Xuxa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>7h45</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Progr(Evandro)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Siste(Eloy)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>Biolo(Debora)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Matem(Silvana)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>8h30</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Lingu(Evandro)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Siste(Eloy)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Geogr(Zeca)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>9h15</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Quimi(Karina)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Artes(Joice)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Geogr(Zeca)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>10h15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PPW(Jessica)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Artes(Joice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>11h00</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PPW(Jessica)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Ed fi(Xuxa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>INTERVALO</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>13h15</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Ed fi(Xuxa)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Desen(Jucemar)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>14h00</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Lingu(Evandro)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Fisic(Felipe)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Socio(Tarso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>14h45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Progr(Evandro)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Socio(Tarso)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>15h45</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Lingu(Evandro)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Quimi(Karina)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Socio(Tarso)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PVIDA(Adriana)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>16h30</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Lingu(Evandro)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Fisic(Felipe)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>7h45</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>PVIDA(Adriana)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Model(Jessica)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Lingu(Evandro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>8h30</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Portu(Marcia)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Matem(Silvana)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Model(Jessica)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Lingu(Evandro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>9h15</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Histo(Walbert)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Desen(Jucemar)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Ed fi(Xuxa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>10h15</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PVIDA(Adriana)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Fisic(Felipe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>11h00</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Siste(Eloy)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PPW(Jessica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>INTERVALO</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>13h15</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Geogr(Zeca)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Socio(Tarso)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Siste(Eloy)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Biolo(Debora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>14h00</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Geogr(Zeca)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Ingle(Natalia)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>PVIDA(Adriana)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>14h45</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Fisic(Felipe)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Progr(Evandro)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Histo(Walbert)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>15h45</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Ed fi(Xuxa)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Histo(Walbert)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Siste(Eloy)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Progr(Evandro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>16h30</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Progr(Evandro)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Biolo(Debora)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Filos(Alex)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Teste(Edilson)</t>
         </is>
       </c>
     </row>

</xml_diff>